<commit_message>
param rhéo kaolin + readme
</commit_message>
<xml_diff>
--- a/Experiences/Mesures kaolin.xlsx
+++ b/Experiences/Mesures kaolin.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Mines IC\TR Fluide\VS\Experiences\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C58654-CC10-42F6-85BC-2974647E3D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C051C1-367F-4D0A-84F3-C4880B9E416A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,21 +25,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>masse goutte</t>
-  </si>
-  <si>
-    <t>D_0</t>
-  </si>
-  <si>
-    <t>D_max</t>
-  </si>
-  <si>
-    <t>masse compression</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>% kaolin</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>m [kg]</t>
+  </si>
+  <si>
+    <t>M [kg]</t>
+  </si>
+  <si>
+    <t>D_0 [mm]</t>
+  </si>
+  <si>
+    <t>D_max [mm]</t>
+  </si>
+  <si>
+    <t>rho [kg/m3]</t>
+  </si>
+  <si>
+    <t>tau0</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>g</t>
   </si>
 </sst>
 </file>
@@ -75,9 +93,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -358,31 +375,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.90625" customWidth="1"/>
+    <col min="2" max="2" width="8.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="5" max="5" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>50</v>
       </c>
@@ -399,8 +438,26 @@
       <c r="E2">
         <v>15.82</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2">
+        <v>1384.1</v>
+      </c>
+      <c r="G2">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H2">
+        <v>7.21</v>
+      </c>
+      <c r="I2">
+        <v>0.79</v>
+      </c>
+      <c r="J2">
+        <v>20237</v>
+      </c>
+      <c r="K2">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>50</v>
       </c>
@@ -417,11 +474,32 @@
       <c r="E3">
         <v>14.14</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3">
+        <v>1384.1</v>
+      </c>
+      <c r="G3">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H3">
+        <v>7.21</v>
+      </c>
+      <c r="I3">
+        <v>0.79</v>
+      </c>
+      <c r="J3">
+        <v>20237</v>
+      </c>
+      <c r="K3">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>50</v>
       </c>
+      <c r="B4">
+        <v>0.08</v>
+      </c>
       <c r="C4">
         <v>20.010100000000001</v>
       </c>
@@ -431,8 +509,26 @@
       <c r="E4">
         <v>10.61</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4">
+        <v>1384.1</v>
+      </c>
+      <c r="G4">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H4">
+        <v>7.21</v>
+      </c>
+      <c r="I4">
+        <v>0.79</v>
+      </c>
+      <c r="J4">
+        <v>20237</v>
+      </c>
+      <c r="K4">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>50</v>
       </c>
@@ -449,8 +545,26 @@
       <c r="E5">
         <v>14.98</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5">
+        <v>1384.1</v>
+      </c>
+      <c r="G5">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H5">
+        <v>7.21</v>
+      </c>
+      <c r="I5">
+        <v>0.79</v>
+      </c>
+      <c r="J5">
+        <v>20237</v>
+      </c>
+      <c r="K5">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>50</v>
       </c>
@@ -467,11 +581,32 @@
       <c r="E6">
         <v>14.66</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6">
+        <v>1384.1</v>
+      </c>
+      <c r="G6">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H6">
+        <v>7.21</v>
+      </c>
+      <c r="I6">
+        <v>0.79</v>
+      </c>
+      <c r="J6">
+        <v>20237</v>
+      </c>
+      <c r="K6">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>50</v>
       </c>
+      <c r="B7">
+        <v>0.1</v>
+      </c>
       <c r="C7">
         <v>100.0247</v>
       </c>
@@ -481,8 +616,26 @@
       <c r="E7">
         <v>16.02</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7">
+        <v>1384.1</v>
+      </c>
+      <c r="G7">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H7">
+        <v>7.21</v>
+      </c>
+      <c r="I7">
+        <v>0.79</v>
+      </c>
+      <c r="J7">
+        <v>20237</v>
+      </c>
+      <c r="K7">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>50</v>
       </c>
@@ -499,11 +652,32 @@
       <c r="E8">
         <v>22.3</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8">
+        <v>1384.1</v>
+      </c>
+      <c r="G8">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H8">
+        <v>7.21</v>
+      </c>
+      <c r="I8">
+        <v>0.79</v>
+      </c>
+      <c r="J8">
+        <v>20237</v>
+      </c>
+      <c r="K8">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>50</v>
       </c>
+      <c r="B9">
+        <v>0.1</v>
+      </c>
       <c r="C9">
         <v>20.010100000000001</v>
       </c>
@@ -513,12 +687,32 @@
       <c r="E9">
         <v>26.04</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9">
+        <v>1384.1</v>
+      </c>
+      <c r="G9">
+        <v>53.235999999999997</v>
+      </c>
+      <c r="H9">
+        <v>7.21</v>
+      </c>
+      <c r="I9">
+        <v>0.79</v>
+      </c>
+      <c r="J9">
+        <v>20237</v>
+      </c>
+      <c r="K9">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>52</v>
       </c>
-      <c r="B10" s="1"/>
+      <c r="B10">
+        <v>7.4999999999999997E-2</v>
+      </c>
       <c r="C10">
         <v>20.010100000000001</v>
       </c>
@@ -528,8 +722,26 @@
       <c r="E10">
         <v>13.62</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10">
+        <v>1450</v>
+      </c>
+      <c r="G10">
+        <v>67.426000000000002</v>
+      </c>
+      <c r="H10">
+        <v>9.15</v>
+      </c>
+      <c r="I10">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="J10">
+        <v>168120</v>
+      </c>
+      <c r="K10">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>52</v>
       </c>
@@ -546,11 +758,32 @@
       <c r="E11">
         <v>11.84</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11">
+        <v>1450</v>
+      </c>
+      <c r="G11">
+        <v>67.426000000000002</v>
+      </c>
+      <c r="H11">
+        <v>9.15</v>
+      </c>
+      <c r="I11">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="J11">
+        <v>168120</v>
+      </c>
+      <c r="K11">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>52</v>
       </c>
+      <c r="B12">
+        <v>7.4999999999999997E-2</v>
+      </c>
       <c r="C12">
         <v>50.121400000000001</v>
       </c>
@@ -560,8 +793,26 @@
       <c r="E12">
         <v>14.9</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12">
+        <v>1450</v>
+      </c>
+      <c r="G12">
+        <v>67.426000000000002</v>
+      </c>
+      <c r="H12">
+        <v>9.15</v>
+      </c>
+      <c r="I12">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="J12">
+        <v>168120</v>
+      </c>
+      <c r="K12">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>52</v>
       </c>
@@ -578,8 +829,26 @@
       <c r="E13">
         <v>15.71</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13">
+        <v>1450</v>
+      </c>
+      <c r="G13">
+        <v>67.426000000000002</v>
+      </c>
+      <c r="H13">
+        <v>9.15</v>
+      </c>
+      <c r="I13">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="J13">
+        <v>168120</v>
+      </c>
+      <c r="K13">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>52</v>
       </c>
@@ -595,6 +864,24 @@
       </c>
       <c r="E14">
         <v>16.38</v>
+      </c>
+      <c r="F14">
+        <v>1450</v>
+      </c>
+      <c r="G14">
+        <v>67.426000000000002</v>
+      </c>
+      <c r="H14">
+        <v>9.15</v>
+      </c>
+      <c r="I14">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="J14">
+        <v>168120</v>
+      </c>
+      <c r="K14">
+        <v>9.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>